<commit_message>
Vérification des blocs : retrait des 63 blocs robots
verification_fonctionnelle_blocs_a_jour.xlsx suit la variante sans
robots : lignes Maqueen Plus, Maqueen Lite, Kitrobot v2 et LiDAR
retirées de l'onglet Blocs (115 blocs), onglet Résumé ajusté (formules
et total), texte des Instructions mis à jour. Résultats de test
inchangés.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/verification_fonctionnelle_blocs_a_jour.xlsx
+++ b/verification_fonctionnelle_blocs_a_jour.xlsx
@@ -13,9 +13,9 @@
     <sheet name="Résumé" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Blocs!$A$1:$I$179</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Blocs!$A$1:$I$116</definedName>
   </definedNames>
-  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
+  <calcPr fullCalcOnLoad="1" iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
@@ -42,7 +42,7 @@
     <t xml:space="preserve">Contenu</t>
   </si>
   <si>
-    <t xml:space="preserve">L'onglet "Blocs" liste les 178 blocs créés pour ce projet (catégorie, sous-catégorie, libellé tel qu'affiché dans la boîte à outils, et identifiant technique interne). Les blocs standards de Blockly (Logique, Boucles natives, Texte, Maths de base, Variables, Fonctions) ne sont pas listés : ce ne sont pas des blocs créés pour ce projet.</t>
+    <t xml:space="preserve">L'onglet "Blocs" liste les 115 blocs créés pour ce projet, variante sans robots (Maqueen Plus, Maqueen Lite, Kitrobot v2 et LiDAR retirés) (catégorie, sous-catégorie, libellé tel qu'affiché dans la boîte à outils, et identifiant technique interne). Les blocs standards de Blockly (Logique, Boucles natives, Texte, Maths de base, Variables, Fonctions) ne sont pas listés : ce ne sont pas des blocs créés pour ce projet.</t>
   </si>
   <si>
     <t xml:space="preserve">Comment remplir</t>
@@ -2275,7 +2275,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I179"/>
+  <dimension ref="A1:I116"/>
   <sheetFormatPr defaultColWidth="8.5625" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
@@ -3483,16 +3483,18 @@
       <c r="H55" s="10"/>
       <c r="I55" s="9"/>
     </row>
-    <row r="56" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="17" t="s">
-        <v>152</v>
-      </c>
-      <c r="B56" s="17"/>
+    <row r="56" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A56" s="21" t="s">
+        <v>282</v>
+      </c>
+      <c r="B56" s="21" t="s">
+        <v>283</v>
+      </c>
       <c r="C56" s="9" t="s">
-        <v>153</v>
+        <v>284</v>
       </c>
       <c r="D56" s="10" t="s">
-        <v>154</v>
+        <v>285</v>
       </c>
       <c r="E56" s="10" t="s">
         <v>36</v>
@@ -3504,16 +3506,18 @@
       <c r="H56" s="10"/>
       <c r="I56" s="9"/>
     </row>
-    <row r="57" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="17" t="s">
-        <v>152</v>
-      </c>
-      <c r="B57" s="17"/>
+    <row r="57" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A57" s="21" t="s">
+        <v>282</v>
+      </c>
+      <c r="B57" s="21" t="s">
+        <v>283</v>
+      </c>
       <c r="C57" s="9" t="s">
-        <v>155</v>
+        <v>286</v>
       </c>
       <c r="D57" s="10" t="s">
-        <v>156</v>
+        <v>287</v>
       </c>
       <c r="E57" s="10" t="s">
         <v>36</v>
@@ -3525,16 +3529,18 @@
       <c r="H57" s="10"/>
       <c r="I57" s="9"/>
     </row>
-    <row r="58" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="17" t="s">
-        <v>152</v>
-      </c>
-      <c r="B58" s="17"/>
+    <row r="58" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A58" s="21" t="s">
+        <v>282</v>
+      </c>
+      <c r="B58" s="21" t="s">
+        <v>288</v>
+      </c>
       <c r="C58" s="9" t="s">
-        <v>157</v>
+        <v>289</v>
       </c>
       <c r="D58" s="10" t="s">
-        <v>158</v>
+        <v>290</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>36</v>
@@ -3547,15 +3553,17 @@
       <c r="I58" s="9"/>
     </row>
     <row r="59" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="17" t="s">
-        <v>152</v>
-      </c>
-      <c r="B59" s="17"/>
+      <c r="A59" s="21" t="s">
+        <v>282</v>
+      </c>
+      <c r="B59" s="21" t="s">
+        <v>288</v>
+      </c>
       <c r="C59" s="9" t="s">
-        <v>159</v>
+        <v>291</v>
       </c>
       <c r="D59" s="10" t="s">
-        <v>160</v>
+        <v>292</v>
       </c>
       <c r="E59" s="10" t="s">
         <v>36</v>
@@ -3568,15 +3576,17 @@
       <c r="I59" s="9"/>
     </row>
     <row r="60" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="17" t="s">
-        <v>152</v>
-      </c>
-      <c r="B60" s="17"/>
+      <c r="A60" s="21" t="s">
+        <v>282</v>
+      </c>
+      <c r="B60" s="21" t="s">
+        <v>288</v>
+      </c>
       <c r="C60" s="9" t="s">
-        <v>161</v>
+        <v>293</v>
       </c>
       <c r="D60" s="10" t="s">
-        <v>162</v>
+        <v>294</v>
       </c>
       <c r="E60" s="10" t="s">
         <v>36</v>
@@ -3589,15 +3599,17 @@
       <c r="I60" s="9"/>
     </row>
     <row r="61" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="17" t="s">
-        <v>152</v>
-      </c>
-      <c r="B61" s="17"/>
+      <c r="A61" s="21" t="s">
+        <v>282</v>
+      </c>
+      <c r="B61" s="21" t="s">
+        <v>288</v>
+      </c>
       <c r="C61" s="9" t="s">
-        <v>163</v>
+        <v>295</v>
       </c>
       <c r="D61" s="10" t="s">
-        <v>164</v>
+        <v>296</v>
       </c>
       <c r="E61" s="10" t="s">
         <v>36</v>
@@ -3610,15 +3622,17 @@
       <c r="I61" s="9"/>
     </row>
     <row r="62" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="17" t="s">
-        <v>152</v>
-      </c>
-      <c r="B62" s="17"/>
+      <c r="A62" s="21" t="s">
+        <v>282</v>
+      </c>
+      <c r="B62" s="21" t="s">
+        <v>288</v>
+      </c>
       <c r="C62" s="9" t="s">
-        <v>165</v>
+        <v>297</v>
       </c>
       <c r="D62" s="10" t="s">
-        <v>166</v>
+        <v>298</v>
       </c>
       <c r="E62" s="10" t="s">
         <v>36</v>
@@ -3630,16 +3644,18 @@
       <c r="H62" s="10"/>
       <c r="I62" s="9"/>
     </row>
-    <row r="63" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A63" s="17" t="s">
-        <v>152</v>
-      </c>
-      <c r="B63" s="17"/>
+    <row r="63" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="21" t="s">
+        <v>282</v>
+      </c>
+      <c r="B63" s="21" t="s">
+        <v>288</v>
+      </c>
       <c r="C63" s="9" t="s">
-        <v>167</v>
+        <v>299</v>
       </c>
       <c r="D63" s="10" t="s">
-        <v>168</v>
+        <v>300</v>
       </c>
       <c r="E63" s="10" t="s">
         <v>36</v>
@@ -3651,16 +3667,18 @@
       <c r="H63" s="10"/>
       <c r="I63" s="9"/>
     </row>
-    <row r="64" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A64" s="17" t="s">
-        <v>152</v>
-      </c>
-      <c r="B64" s="17"/>
+    <row r="64" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="21" t="s">
+        <v>282</v>
+      </c>
+      <c r="B64" s="21" t="s">
+        <v>288</v>
+      </c>
       <c r="C64" s="9" t="s">
-        <v>169</v>
+        <v>301</v>
       </c>
       <c r="D64" s="10" t="s">
-        <v>170</v>
+        <v>302</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>36</v>
@@ -3672,16 +3690,18 @@
       <c r="H64" s="10"/>
       <c r="I64" s="9"/>
     </row>
-    <row r="65" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A65" s="17" t="s">
-        <v>152</v>
-      </c>
-      <c r="B65" s="17"/>
+    <row r="65" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="21" t="s">
+        <v>282</v>
+      </c>
+      <c r="B65" s="21" t="s">
+        <v>288</v>
+      </c>
       <c r="C65" s="9" t="s">
-        <v>171</v>
+        <v>303</v>
       </c>
       <c r="D65" s="10" t="s">
-        <v>172</v>
+        <v>304</v>
       </c>
       <c r="E65" s="10" t="s">
         <v>36</v>
@@ -3693,16 +3713,18 @@
       <c r="H65" s="10"/>
       <c r="I65" s="9"/>
     </row>
-    <row r="66" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A66" s="17" t="s">
-        <v>152</v>
-      </c>
-      <c r="B66" s="17"/>
+    <row r="66" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="21" t="s">
+        <v>282</v>
+      </c>
+      <c r="B66" s="21" t="s">
+        <v>305</v>
+      </c>
       <c r="C66" s="9" t="s">
-        <v>173</v>
+        <v>306</v>
       </c>
       <c r="D66" s="10" t="s">
-        <v>174</v>
+        <v>307</v>
       </c>
       <c r="E66" s="10" t="s">
         <v>36</v>
@@ -3714,16 +3736,18 @@
       <c r="H66" s="10"/>
       <c r="I66" s="9"/>
     </row>
-    <row r="67" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A67" s="17" t="s">
-        <v>152</v>
-      </c>
-      <c r="B67" s="17"/>
+    <row r="67" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="21" t="s">
+        <v>282</v>
+      </c>
+      <c r="B67" s="21" t="s">
+        <v>305</v>
+      </c>
       <c r="C67" s="9" t="s">
-        <v>175</v>
+        <v>308</v>
       </c>
       <c r="D67" s="10" t="s">
-        <v>176</v>
+        <v>309</v>
       </c>
       <c r="E67" s="10" t="s">
         <v>36</v>
@@ -3735,16 +3759,18 @@
       <c r="H67" s="10"/>
       <c r="I67" s="9"/>
     </row>
-    <row r="68" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A68" s="17" t="s">
-        <v>152</v>
-      </c>
-      <c r="B68" s="17"/>
+    <row r="68" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="21" t="s">
+        <v>282</v>
+      </c>
+      <c r="B68" s="21" t="s">
+        <v>305</v>
+      </c>
       <c r="C68" s="9" t="s">
-        <v>177</v>
+        <v>310</v>
       </c>
       <c r="D68" s="10" t="s">
-        <v>178</v>
+        <v>311</v>
       </c>
       <c r="E68" s="10" t="s">
         <v>36</v>
@@ -3757,15 +3783,17 @@
       <c r="I68" s="9"/>
     </row>
     <row r="69" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="17" t="s">
-        <v>152</v>
-      </c>
-      <c r="B69" s="17"/>
+      <c r="A69" s="21" t="s">
+        <v>282</v>
+      </c>
+      <c r="B69" s="21" t="s">
+        <v>305</v>
+      </c>
       <c r="C69" s="9" t="s">
-        <v>179</v>
+        <v>312</v>
       </c>
       <c r="D69" s="10" t="s">
-        <v>180</v>
+        <v>313</v>
       </c>
       <c r="E69" s="10" t="s">
         <v>36</v>
@@ -3777,16 +3805,18 @@
       <c r="H69" s="10"/>
       <c r="I69" s="9"/>
     </row>
-    <row r="70" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A70" s="17" t="s">
-        <v>152</v>
-      </c>
-      <c r="B70" s="17"/>
+    <row r="70" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="21" t="s">
+        <v>282</v>
+      </c>
+      <c r="B70" s="21" t="s">
+        <v>305</v>
+      </c>
       <c r="C70" s="9" t="s">
-        <v>181</v>
+        <v>314</v>
       </c>
       <c r="D70" s="10" t="s">
-        <v>182</v>
+        <v>315</v>
       </c>
       <c r="E70" s="10" t="s">
         <v>36</v>
@@ -3798,16 +3828,18 @@
       <c r="H70" s="10"/>
       <c r="I70" s="9"/>
     </row>
-    <row r="71" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A71" s="17" t="s">
-        <v>152</v>
-      </c>
-      <c r="B71" s="17"/>
+    <row r="71" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="21" t="s">
+        <v>282</v>
+      </c>
+      <c r="B71" s="21" t="s">
+        <v>305</v>
+      </c>
       <c r="C71" s="9" t="s">
-        <v>183</v>
+        <v>316</v>
       </c>
       <c r="D71" s="10" t="s">
-        <v>184</v>
+        <v>317</v>
       </c>
       <c r="E71" s="10" t="s">
         <v>36</v>
@@ -3820,15 +3852,17 @@
       <c r="I71" s="9"/>
     </row>
     <row r="72" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="17" t="s">
-        <v>152</v>
-      </c>
-      <c r="B72" s="17"/>
+      <c r="A72" s="21" t="s">
+        <v>282</v>
+      </c>
+      <c r="B72" s="21" t="s">
+        <v>318</v>
+      </c>
       <c r="C72" s="9" t="s">
-        <v>185</v>
+        <v>319</v>
       </c>
       <c r="D72" s="10" t="s">
-        <v>186</v>
+        <v>320</v>
       </c>
       <c r="E72" s="10" t="s">
         <v>36</v>
@@ -3840,16 +3874,18 @@
       <c r="H72" s="10"/>
       <c r="I72" s="9"/>
     </row>
-    <row r="73" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A73" s="17" t="s">
-        <v>152</v>
-      </c>
-      <c r="B73" s="17"/>
+    <row r="73" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="21" t="s">
+        <v>282</v>
+      </c>
+      <c r="B73" s="21" t="s">
+        <v>318</v>
+      </c>
       <c r="C73" s="9" t="s">
-        <v>187</v>
+        <v>321</v>
       </c>
       <c r="D73" s="10" t="s">
-        <v>188</v>
+        <v>322</v>
       </c>
       <c r="E73" s="10" t="s">
         <v>36</v>
@@ -3861,16 +3897,18 @@
       <c r="H73" s="10"/>
       <c r="I73" s="9"/>
     </row>
-    <row r="74" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A74" s="17" t="s">
-        <v>152</v>
-      </c>
-      <c r="B74" s="17"/>
+    <row r="74" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="21" t="s">
+        <v>282</v>
+      </c>
+      <c r="B74" s="21" t="s">
+        <v>323</v>
+      </c>
       <c r="C74" s="9" t="s">
-        <v>189</v>
+        <v>324</v>
       </c>
       <c r="D74" s="10" t="s">
-        <v>190</v>
+        <v>325</v>
       </c>
       <c r="E74" s="10" t="s">
         <v>36</v>
@@ -3882,16 +3920,18 @@
       <c r="H74" s="10"/>
       <c r="I74" s="9"/>
     </row>
-    <row r="75" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A75" s="17" t="s">
-        <v>152</v>
-      </c>
-      <c r="B75" s="17"/>
+    <row r="75" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A75" s="21" t="s">
+        <v>282</v>
+      </c>
+      <c r="B75" s="21" t="s">
+        <v>323</v>
+      </c>
       <c r="C75" s="9" t="s">
-        <v>191</v>
+        <v>326</v>
       </c>
       <c r="D75" s="10" t="s">
-        <v>192</v>
+        <v>327</v>
       </c>
       <c r="E75" s="10" t="s">
         <v>36</v>
@@ -3903,16 +3943,18 @@
       <c r="H75" s="10"/>
       <c r="I75" s="9"/>
     </row>
-    <row r="76" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A76" s="17" t="s">
-        <v>152</v>
-      </c>
-      <c r="B76" s="17"/>
+    <row r="76" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A76" s="21" t="s">
+        <v>282</v>
+      </c>
+      <c r="B76" s="21" t="s">
+        <v>323</v>
+      </c>
       <c r="C76" s="9" t="s">
-        <v>193</v>
+        <v>328</v>
       </c>
       <c r="D76" s="10" t="s">
-        <v>194</v>
+        <v>329</v>
       </c>
       <c r="E76" s="10" t="s">
         <v>36</v>
@@ -3924,16 +3966,18 @@
       <c r="H76" s="10"/>
       <c r="I76" s="9"/>
     </row>
-    <row r="77" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A77" s="17" t="s">
-        <v>152</v>
-      </c>
-      <c r="B77" s="17"/>
+    <row r="77" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A77" s="21" t="s">
+        <v>282</v>
+      </c>
+      <c r="B77" s="21" t="s">
+        <v>330</v>
+      </c>
       <c r="C77" s="9" t="s">
-        <v>195</v>
+        <v>331</v>
       </c>
       <c r="D77" s="10" t="s">
-        <v>196</v>
+        <v>332</v>
       </c>
       <c r="E77" s="10" t="s">
         <v>36</v>
@@ -3945,16 +3989,18 @@
       <c r="H77" s="10"/>
       <c r="I77" s="9"/>
     </row>
-    <row r="78" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A78" s="17" t="s">
-        <v>152</v>
-      </c>
-      <c r="B78" s="17"/>
+    <row r="78" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A78" s="21" t="s">
+        <v>282</v>
+      </c>
+      <c r="B78" s="21" t="s">
+        <v>330</v>
+      </c>
       <c r="C78" s="9" t="s">
-        <v>197</v>
+        <v>333</v>
       </c>
       <c r="D78" s="10" t="s">
-        <v>198</v>
+        <v>334</v>
       </c>
       <c r="E78" s="10" t="s">
         <v>36</v>
@@ -3966,16 +4012,18 @@
       <c r="H78" s="10"/>
       <c r="I78" s="9"/>
     </row>
-    <row r="79" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A79" s="17" t="s">
-        <v>152</v>
-      </c>
-      <c r="B79" s="17"/>
+    <row r="79" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A79" s="21" t="s">
+        <v>282</v>
+      </c>
+      <c r="B79" s="21" t="s">
+        <v>330</v>
+      </c>
       <c r="C79" s="9" t="s">
-        <v>199</v>
+        <v>335</v>
       </c>
       <c r="D79" s="10" t="s">
-        <v>200</v>
+        <v>336</v>
       </c>
       <c r="E79" s="10" t="s">
         <v>36</v>
@@ -3988,15 +4036,17 @@
       <c r="I79" s="9"/>
     </row>
     <row r="80" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A80" s="17" t="s">
-        <v>152</v>
-      </c>
-      <c r="B80" s="17"/>
+      <c r="A80" s="21" t="s">
+        <v>282</v>
+      </c>
+      <c r="B80" s="21" t="s">
+        <v>337</v>
+      </c>
       <c r="C80" s="9" t="s">
-        <v>201</v>
+        <v>338</v>
       </c>
       <c r="D80" s="10" t="s">
-        <v>202</v>
+        <v>339</v>
       </c>
       <c r="E80" s="10" t="s">
         <v>36</v>
@@ -4008,16 +4058,18 @@
       <c r="H80" s="10"/>
       <c r="I80" s="9"/>
     </row>
-    <row r="81" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A81" s="17" t="s">
-        <v>152</v>
-      </c>
-      <c r="B81" s="17"/>
+    <row r="81" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A81" s="21" t="s">
+        <v>282</v>
+      </c>
+      <c r="B81" s="21" t="s">
+        <v>337</v>
+      </c>
       <c r="C81" s="9" t="s">
-        <v>203</v>
+        <v>340</v>
       </c>
       <c r="D81" s="10" t="s">
-        <v>204</v>
+        <v>341</v>
       </c>
       <c r="E81" s="10" t="s">
         <v>36</v>
@@ -4029,16 +4081,18 @@
       <c r="H81" s="10"/>
       <c r="I81" s="9"/>
     </row>
-    <row r="82" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A82" s="17" t="s">
-        <v>152</v>
-      </c>
-      <c r="B82" s="17"/>
+    <row r="82" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A82" s="21" t="s">
+        <v>282</v>
+      </c>
+      <c r="B82" s="21" t="s">
+        <v>337</v>
+      </c>
       <c r="C82" s="9" t="s">
-        <v>205</v>
+        <v>342</v>
       </c>
       <c r="D82" s="10" t="s">
-        <v>206</v>
+        <v>343</v>
       </c>
       <c r="E82" s="10" t="s">
         <v>36</v>
@@ -4050,16 +4104,18 @@
       <c r="H82" s="10"/>
       <c r="I82" s="9"/>
     </row>
-    <row r="83" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A83" s="18" t="s">
-        <v>207</v>
-      </c>
-      <c r="B83" s="18"/>
+    <row r="83" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A83" s="21" t="s">
+        <v>282</v>
+      </c>
+      <c r="B83" s="21" t="s">
+        <v>337</v>
+      </c>
       <c r="C83" s="9" t="s">
-        <v>208</v>
+        <v>344</v>
       </c>
       <c r="D83" s="10" t="s">
-        <v>209</v>
+        <v>345</v>
       </c>
       <c r="E83" s="10" t="s">
         <v>36</v>
@@ -4072,15 +4128,17 @@
       <c r="I83" s="9"/>
     </row>
     <row r="84" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A84" s="18" t="s">
-        <v>207</v>
-      </c>
-      <c r="B84" s="18"/>
+      <c r="A84" s="21" t="s">
+        <v>282</v>
+      </c>
+      <c r="B84" s="21" t="s">
+        <v>337</v>
+      </c>
       <c r="C84" s="9" t="s">
-        <v>210</v>
+        <v>346</v>
       </c>
       <c r="D84" s="10" t="s">
-        <v>211</v>
+        <v>347</v>
       </c>
       <c r="E84" s="10" t="s">
         <v>36</v>
@@ -4092,16 +4150,18 @@
       <c r="H84" s="10"/>
       <c r="I84" s="9"/>
     </row>
-    <row r="85" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A85" s="18" t="s">
-        <v>207</v>
-      </c>
-      <c r="B85" s="18"/>
+    <row r="85" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A85" s="21" t="s">
+        <v>282</v>
+      </c>
+      <c r="B85" s="21" t="s">
+        <v>337</v>
+      </c>
       <c r="C85" s="9" t="s">
-        <v>212</v>
+        <v>348</v>
       </c>
       <c r="D85" s="10" t="s">
-        <v>213</v>
+        <v>349</v>
       </c>
       <c r="E85" s="10" t="s">
         <v>36</v>
@@ -4113,100 +4173,110 @@
       <c r="H85" s="10"/>
       <c r="I85" s="9"/>
     </row>
-    <row r="86" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A86" s="18" t="s">
-        <v>207</v>
-      </c>
-      <c r="B86" s="18"/>
+    <row r="86" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A86" s="21" t="s">
+        <v>282</v>
+      </c>
+      <c r="B86" s="21" t="s">
+        <v>350</v>
+      </c>
       <c r="C86" s="9" t="s">
-        <v>214</v>
+        <v>351</v>
       </c>
       <c r="D86" s="10" t="s">
-        <v>215</v>
+        <v>352</v>
       </c>
       <c r="E86" s="10" t="s">
-        <v>36</v>
+        <v>23</v>
       </c>
       <c r="F86" s="10" t="s">
-        <v>36</v>
+        <v>23</v>
       </c>
       <c r="G86" s="10"/>
       <c r="H86" s="10"/>
       <c r="I86" s="9"/>
     </row>
-    <row r="87" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A87" s="18" t="s">
-        <v>207</v>
-      </c>
-      <c r="B87" s="18"/>
+    <row r="87" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A87" s="21" t="s">
+        <v>282</v>
+      </c>
+      <c r="B87" s="21" t="s">
+        <v>350</v>
+      </c>
       <c r="C87" s="9" t="s">
-        <v>216</v>
+        <v>353</v>
       </c>
       <c r="D87" s="10" t="s">
-        <v>217</v>
+        <v>354</v>
       </c>
       <c r="E87" s="10" t="s">
-        <v>36</v>
+        <v>23</v>
       </c>
       <c r="F87" s="10" t="s">
-        <v>36</v>
+        <v>23</v>
       </c>
       <c r="G87" s="10"/>
       <c r="H87" s="10"/>
       <c r="I87" s="9"/>
     </row>
     <row r="88" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A88" s="18" t="s">
-        <v>207</v>
-      </c>
-      <c r="B88" s="18"/>
+      <c r="A88" s="21" t="s">
+        <v>282</v>
+      </c>
+      <c r="B88" s="21" t="s">
+        <v>350</v>
+      </c>
       <c r="C88" s="9" t="s">
-        <v>218</v>
+        <v>355</v>
       </c>
       <c r="D88" s="10" t="s">
-        <v>219</v>
+        <v>356</v>
       </c>
       <c r="E88" s="10" t="s">
-        <v>36</v>
+        <v>23</v>
       </c>
       <c r="F88" s="10" t="s">
-        <v>36</v>
+        <v>23</v>
       </c>
       <c r="G88" s="10"/>
       <c r="H88" s="10"/>
       <c r="I88" s="9"/>
     </row>
     <row r="89" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A89" s="18" t="s">
-        <v>207</v>
-      </c>
-      <c r="B89" s="18"/>
+      <c r="A89" s="21" t="s">
+        <v>282</v>
+      </c>
+      <c r="B89" s="21" t="s">
+        <v>350</v>
+      </c>
       <c r="C89" s="9" t="s">
-        <v>220</v>
+        <v>357</v>
       </c>
       <c r="D89" s="10" t="s">
-        <v>221</v>
+        <v>358</v>
       </c>
       <c r="E89" s="10" t="s">
-        <v>36</v>
+        <v>23</v>
       </c>
       <c r="F89" s="10" t="s">
-        <v>36</v>
+        <v>359</v>
       </c>
       <c r="G89" s="10"/>
       <c r="H89" s="10"/>
       <c r="I89" s="9"/>
     </row>
     <row r="90" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A90" s="19" t="s">
-        <v>222</v>
-      </c>
-      <c r="B90" s="19"/>
+      <c r="A90" s="21" t="s">
+        <v>282</v>
+      </c>
+      <c r="B90" s="21" t="s">
+        <v>360</v>
+      </c>
       <c r="C90" s="9" t="s">
-        <v>223</v>
+        <v>361</v>
       </c>
       <c r="D90" s="10" t="s">
-        <v>224</v>
+        <v>362</v>
       </c>
       <c r="E90" s="10" t="s">
         <v>36</v>
@@ -4219,15 +4289,17 @@
       <c r="I90" s="9"/>
     </row>
     <row r="91" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A91" s="19" t="s">
-        <v>222</v>
-      </c>
-      <c r="B91" s="19"/>
+      <c r="A91" s="21" t="s">
+        <v>282</v>
+      </c>
+      <c r="B91" s="21" t="s">
+        <v>360</v>
+      </c>
       <c r="C91" s="9" t="s">
-        <v>225</v>
+        <v>363</v>
       </c>
       <c r="D91" s="10" t="s">
-        <v>226</v>
+        <v>364</v>
       </c>
       <c r="E91" s="10" t="s">
         <v>36</v>
@@ -4240,15 +4312,17 @@
       <c r="I91" s="9"/>
     </row>
     <row r="92" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A92" s="19" t="s">
-        <v>222</v>
-      </c>
-      <c r="B92" s="19"/>
+      <c r="A92" s="21" t="s">
+        <v>282</v>
+      </c>
+      <c r="B92" s="21" t="s">
+        <v>365</v>
+      </c>
       <c r="C92" s="9" t="s">
-        <v>227</v>
+        <v>366</v>
       </c>
       <c r="D92" s="10" t="s">
-        <v>228</v>
+        <v>367</v>
       </c>
       <c r="E92" s="10" t="s">
         <v>36</v>
@@ -4260,16 +4334,18 @@
       <c r="H92" s="10"/>
       <c r="I92" s="9"/>
     </row>
-    <row r="93" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A93" s="19" t="s">
-        <v>222</v>
-      </c>
-      <c r="B93" s="19"/>
+    <row r="93" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A93" s="21" t="s">
+        <v>282</v>
+      </c>
+      <c r="B93" s="21" t="s">
+        <v>365</v>
+      </c>
       <c r="C93" s="9" t="s">
-        <v>229</v>
+        <v>368</v>
       </c>
       <c r="D93" s="10" t="s">
-        <v>230</v>
+        <v>369</v>
       </c>
       <c r="E93" s="10" t="s">
         <v>36</v>
@@ -4281,16 +4357,18 @@
       <c r="H93" s="10"/>
       <c r="I93" s="9"/>
     </row>
-    <row r="94" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A94" s="19" t="s">
-        <v>222</v>
-      </c>
-      <c r="B94" s="19"/>
+    <row r="94" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A94" s="21" t="s">
+        <v>282</v>
+      </c>
+      <c r="B94" s="21" t="s">
+        <v>365</v>
+      </c>
       <c r="C94" s="9" t="s">
-        <v>231</v>
+        <v>370</v>
       </c>
       <c r="D94" s="10" t="s">
-        <v>232</v>
+        <v>371</v>
       </c>
       <c r="E94" s="10" t="s">
         <v>36</v>
@@ -4303,15 +4381,17 @@
       <c r="I94" s="9"/>
     </row>
     <row r="95" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A95" s="19" t="s">
-        <v>222</v>
-      </c>
-      <c r="B95" s="19"/>
+      <c r="A95" s="21" t="s">
+        <v>282</v>
+      </c>
+      <c r="B95" s="21" t="s">
+        <v>372</v>
+      </c>
       <c r="C95" s="9" t="s">
-        <v>233</v>
+        <v>373</v>
       </c>
       <c r="D95" s="10" t="s">
-        <v>234</v>
+        <v>374</v>
       </c>
       <c r="E95" s="10" t="s">
         <v>36</v>
@@ -4324,15 +4404,17 @@
       <c r="I95" s="9"/>
     </row>
     <row r="96" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A96" s="19" t="s">
-        <v>222</v>
-      </c>
-      <c r="B96" s="19"/>
+      <c r="A96" s="21" t="s">
+        <v>282</v>
+      </c>
+      <c r="B96" s="21" t="s">
+        <v>372</v>
+      </c>
       <c r="C96" s="9" t="s">
-        <v>235</v>
+        <v>375</v>
       </c>
       <c r="D96" s="10" t="s">
-        <v>236</v>
+        <v>376</v>
       </c>
       <c r="E96" s="10" t="s">
         <v>36</v>
@@ -4345,15 +4427,17 @@
       <c r="I96" s="9"/>
     </row>
     <row r="97" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A97" s="19" t="s">
-        <v>222</v>
-      </c>
-      <c r="B97" s="19"/>
+      <c r="A97" s="21" t="s">
+        <v>282</v>
+      </c>
+      <c r="B97" s="21" t="s">
+        <v>372</v>
+      </c>
       <c r="C97" s="9" t="s">
-        <v>237</v>
+        <v>377</v>
       </c>
       <c r="D97" s="10" t="s">
-        <v>238</v>
+        <v>378</v>
       </c>
       <c r="E97" s="10" t="s">
         <v>36</v>
@@ -4366,15 +4450,17 @@
       <c r="I97" s="9"/>
     </row>
     <row r="98" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A98" s="19" t="s">
-        <v>222</v>
-      </c>
-      <c r="B98" s="19"/>
+      <c r="A98" s="21" t="s">
+        <v>282</v>
+      </c>
+      <c r="B98" s="21" t="s">
+        <v>372</v>
+      </c>
       <c r="C98" s="9" t="s">
-        <v>239</v>
+        <v>379</v>
       </c>
       <c r="D98" s="10" t="s">
-        <v>240</v>
+        <v>380</v>
       </c>
       <c r="E98" s="10" t="s">
         <v>36</v>
@@ -4386,16 +4472,16 @@
       <c r="H98" s="10"/>
       <c r="I98" s="9"/>
     </row>
-    <row r="99" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A99" s="19" t="s">
-        <v>222</v>
-      </c>
-      <c r="B99" s="19"/>
+    <row r="99" customFormat="false" ht="35.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A99" s="21" t="s">
+        <v>282</v>
+      </c>
+      <c r="B99" s="21"/>
       <c r="C99" s="9" t="s">
-        <v>241</v>
+        <v>381</v>
       </c>
       <c r="D99" s="10" t="s">
-        <v>242</v>
+        <v>382</v>
       </c>
       <c r="E99" s="10" t="s">
         <v>36</v>
@@ -4405,18 +4491,20 @@
       </c>
       <c r="G99" s="10"/>
       <c r="H99" s="10"/>
-      <c r="I99" s="9"/>
+      <c r="I99" s="9" t="s">
+        <v>383</v>
+      </c>
     </row>
     <row r="100" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A100" s="19" t="s">
-        <v>222</v>
-      </c>
-      <c r="B100" s="19"/>
+      <c r="A100" s="21" t="s">
+        <v>282</v>
+      </c>
+      <c r="B100" s="21"/>
       <c r="C100" s="9" t="s">
-        <v>243</v>
+        <v>384</v>
       </c>
       <c r="D100" s="10" t="s">
-        <v>244</v>
+        <v>385</v>
       </c>
       <c r="E100" s="10" t="s">
         <v>36</v>
@@ -4426,18 +4514,20 @@
       </c>
       <c r="G100" s="10"/>
       <c r="H100" s="10"/>
-      <c r="I100" s="9"/>
+      <c r="I100" s="9" t="s">
+        <v>386</v>
+      </c>
     </row>
     <row r="101" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A101" s="19" t="s">
-        <v>222</v>
-      </c>
-      <c r="B101" s="19"/>
+      <c r="A101" s="21" t="s">
+        <v>282</v>
+      </c>
+      <c r="B101" s="21"/>
       <c r="C101" s="9" t="s">
-        <v>245</v>
+        <v>387</v>
       </c>
       <c r="D101" s="10" t="s">
-        <v>246</v>
+        <v>388</v>
       </c>
       <c r="E101" s="10" t="s">
         <v>36</v>
@@ -4449,16 +4539,16 @@
       <c r="H101" s="10"/>
       <c r="I101" s="9"/>
     </row>
-    <row r="102" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A102" s="19" t="s">
-        <v>222</v>
-      </c>
-      <c r="B102" s="19"/>
+    <row r="102" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A102" s="21" t="s">
+        <v>282</v>
+      </c>
+      <c r="B102" s="21"/>
       <c r="C102" s="9" t="s">
-        <v>247</v>
+        <v>389</v>
       </c>
       <c r="D102" s="10" t="s">
-        <v>248</v>
+        <v>390</v>
       </c>
       <c r="E102" s="10" t="s">
         <v>36</v>
@@ -4468,18 +4558,20 @@
       </c>
       <c r="G102" s="10"/>
       <c r="H102" s="10"/>
-      <c r="I102" s="9"/>
-    </row>
-    <row r="103" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A103" s="19" t="s">
-        <v>222</v>
-      </c>
-      <c r="B103" s="19"/>
+      <c r="I102" s="9" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="103" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A103" s="21" t="s">
+        <v>282</v>
+      </c>
+      <c r="B103" s="21"/>
       <c r="C103" s="9" t="s">
-        <v>249</v>
+        <v>392</v>
       </c>
       <c r="D103" s="10" t="s">
-        <v>250</v>
+        <v>393</v>
       </c>
       <c r="E103" s="10" t="s">
         <v>36</v>
@@ -4489,18 +4581,20 @@
       </c>
       <c r="G103" s="10"/>
       <c r="H103" s="10"/>
-      <c r="I103" s="9"/>
-    </row>
-    <row r="104" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A104" s="19" t="s">
-        <v>222</v>
-      </c>
-      <c r="B104" s="19"/>
+      <c r="I103" s="9" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="104" customFormat="false" ht="35.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A104" s="21" t="s">
+        <v>282</v>
+      </c>
+      <c r="B104" s="21"/>
       <c r="C104" s="9" t="s">
-        <v>251</v>
+        <v>395</v>
       </c>
       <c r="D104" s="10" t="s">
-        <v>252</v>
+        <v>396</v>
       </c>
       <c r="E104" s="10" t="s">
         <v>36</v>
@@ -4510,18 +4604,20 @@
       </c>
       <c r="G104" s="10"/>
       <c r="H104" s="10"/>
-      <c r="I104" s="9"/>
-    </row>
-    <row r="105" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A105" s="19" t="s">
-        <v>222</v>
-      </c>
-      <c r="B105" s="19"/>
+      <c r="I104" s="9" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="105" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A105" s="21" t="s">
+        <v>282</v>
+      </c>
+      <c r="B105" s="21"/>
       <c r="C105" s="9" t="s">
-        <v>253</v>
+        <v>398</v>
       </c>
       <c r="D105" s="10" t="s">
-        <v>254</v>
+        <v>399</v>
       </c>
       <c r="E105" s="10" t="s">
         <v>36</v>
@@ -4531,18 +4627,20 @@
       </c>
       <c r="G105" s="10"/>
       <c r="H105" s="10"/>
-      <c r="I105" s="9"/>
-    </row>
-    <row r="106" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A106" s="19" t="s">
-        <v>222</v>
-      </c>
-      <c r="B106" s="19"/>
+      <c r="I105" s="9" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="106" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A106" s="22" t="s">
+        <v>401</v>
+      </c>
+      <c r="B106" s="22"/>
       <c r="C106" s="9" t="s">
-        <v>255</v>
+        <v>402</v>
       </c>
       <c r="D106" s="10" t="s">
-        <v>256</v>
+        <v>403</v>
       </c>
       <c r="E106" s="10" t="s">
         <v>36</v>
@@ -4555,15 +4653,15 @@
       <c r="I106" s="9"/>
     </row>
     <row r="107" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A107" s="19" t="s">
-        <v>222</v>
-      </c>
-      <c r="B107" s="19"/>
+      <c r="A107" s="22" t="s">
+        <v>401</v>
+      </c>
+      <c r="B107" s="22"/>
       <c r="C107" s="9" t="s">
-        <v>257</v>
+        <v>404</v>
       </c>
       <c r="D107" s="10" t="s">
-        <v>258</v>
+        <v>405</v>
       </c>
       <c r="E107" s="10" t="s">
         <v>36</v>
@@ -4575,16 +4673,16 @@
       <c r="H107" s="10"/>
       <c r="I107" s="9"/>
     </row>
-    <row r="108" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A108" s="19" t="s">
-        <v>222</v>
-      </c>
-      <c r="B108" s="19"/>
+    <row r="108" customFormat="false" ht="52.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A108" s="23" t="s">
+        <v>406</v>
+      </c>
+      <c r="B108" s="23"/>
       <c r="C108" s="9" t="s">
-        <v>259</v>
+        <v>407</v>
       </c>
       <c r="D108" s="10" t="s">
-        <v>260</v>
+        <v>408</v>
       </c>
       <c r="E108" s="10" t="s">
         <v>36</v>
@@ -4596,16 +4694,16 @@
       <c r="H108" s="10"/>
       <c r="I108" s="9"/>
     </row>
-    <row r="109" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A109" s="19" t="s">
-        <v>222</v>
-      </c>
-      <c r="B109" s="19"/>
+    <row r="109" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A109" s="23" t="s">
+        <v>406</v>
+      </c>
+      <c r="B109" s="23"/>
       <c r="C109" s="9" t="s">
-        <v>261</v>
+        <v>409</v>
       </c>
       <c r="D109" s="10" t="s">
-        <v>262</v>
+        <v>410</v>
       </c>
       <c r="E109" s="10" t="s">
         <v>36</v>
@@ -4618,15 +4716,13 @@
       <c r="I109" s="9"/>
     </row>
     <row r="110" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A110" s="19" t="s">
-        <v>222</v>
-      </c>
-      <c r="B110" s="19"/>
-      <c r="C110" s="9" t="s">
-        <v>263</v>
-      </c>
+      <c r="A110" s="23" t="s">
+        <v>406</v>
+      </c>
+      <c r="B110" s="23"/>
+      <c r="C110" s="9"/>
       <c r="D110" s="10" t="s">
-        <v>264</v>
+        <v>411</v>
       </c>
       <c r="E110" s="10" t="s">
         <v>36</v>
@@ -4639,36 +4735,34 @@
       <c r="I110" s="9"/>
     </row>
     <row r="111" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A111" s="20" t="s">
-        <v>265</v>
-      </c>
-      <c r="B111" s="20"/>
-      <c r="C111" s="9" t="s">
-        <v>266</v>
-      </c>
+      <c r="A111" s="23" t="s">
+        <v>406</v>
+      </c>
+      <c r="B111" s="23"/>
+      <c r="C111" s="9"/>
       <c r="D111" s="10" t="s">
-        <v>267</v>
+        <v>412</v>
       </c>
       <c r="E111" s="10" t="s">
-        <v>36</v>
+        <v>23</v>
       </c>
       <c r="F111" s="10" t="s">
-        <v>36</v>
+        <v>23</v>
       </c>
       <c r="G111" s="10"/>
       <c r="H111" s="10"/>
       <c r="I111" s="9"/>
     </row>
-    <row r="112" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A112" s="20" t="s">
-        <v>265</v>
-      </c>
-      <c r="B112" s="20"/>
+    <row r="112" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A112" s="23" t="s">
+        <v>406</v>
+      </c>
+      <c r="B112" s="23"/>
       <c r="C112" s="9" t="s">
-        <v>268</v>
+        <v>413</v>
       </c>
       <c r="D112" s="10" t="s">
-        <v>269</v>
+        <v>414</v>
       </c>
       <c r="E112" s="10" t="s">
         <v>36</v>
@@ -4680,16 +4774,16 @@
       <c r="H112" s="10"/>
       <c r="I112" s="9"/>
     </row>
-    <row r="113" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A113" s="20" t="s">
-        <v>265</v>
-      </c>
-      <c r="B113" s="20"/>
+    <row r="113" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A113" s="23" t="s">
+        <v>406</v>
+      </c>
+      <c r="B113" s="23"/>
       <c r="C113" s="9" t="s">
-        <v>270</v>
+        <v>415</v>
       </c>
       <c r="D113" s="10" t="s">
-        <v>271</v>
+        <v>416</v>
       </c>
       <c r="E113" s="10" t="s">
         <v>36</v>
@@ -4701,16 +4795,16 @@
       <c r="H113" s="10"/>
       <c r="I113" s="9"/>
     </row>
-    <row r="114" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A114" s="20" t="s">
-        <v>265</v>
-      </c>
-      <c r="B114" s="20"/>
+    <row r="114" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A114" s="23" t="s">
+        <v>406</v>
+      </c>
+      <c r="B114" s="23"/>
       <c r="C114" s="9" t="s">
-        <v>272</v>
+        <v>417</v>
       </c>
       <c r="D114" s="10" t="s">
-        <v>273</v>
+        <v>418</v>
       </c>
       <c r="E114" s="10" t="s">
         <v>36</v>
@@ -4722,16 +4816,18 @@
       <c r="H114" s="10"/>
       <c r="I114" s="9"/>
     </row>
-    <row r="115" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A115" s="20" t="s">
-        <v>265</v>
-      </c>
-      <c r="B115" s="20"/>
+    <row r="115" customFormat="false" ht="46.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A115" s="24" t="s">
+        <v>419</v>
+      </c>
+      <c r="B115" s="23" t="s">
+        <v>420</v>
+      </c>
       <c r="C115" s="9" t="s">
-        <v>274</v>
+        <v>421</v>
       </c>
       <c r="D115" s="10" t="s">
-        <v>275</v>
+        <v>422</v>
       </c>
       <c r="E115" s="10" t="s">
         <v>36</v>
@@ -4741,18 +4837,22 @@
       </c>
       <c r="G115" s="10"/>
       <c r="H115" s="10"/>
-      <c r="I115" s="9"/>
-    </row>
-    <row r="116" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A116" s="20" t="s">
-        <v>265</v>
-      </c>
-      <c r="B116" s="20"/>
+      <c r="I115" s="9" t="s">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="116" customFormat="false" ht="35.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A116" s="24" t="s">
+        <v>419</v>
+      </c>
+      <c r="B116" s="23" t="s">
+        <v>424</v>
+      </c>
       <c r="C116" s="9" t="s">
-        <v>276</v>
+        <v>425</v>
       </c>
       <c r="D116" s="10" t="s">
-        <v>277</v>
+        <v>426</v>
       </c>
       <c r="E116" s="10" t="s">
         <v>36</v>
@@ -4762,1437 +4862,14 @@
       </c>
       <c r="G116" s="10"/>
       <c r="H116" s="10"/>
-      <c r="I116" s="9"/>
-    </row>
-    <row r="117" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A117" s="20" t="s">
-        <v>265</v>
-      </c>
-      <c r="B117" s="20"/>
-      <c r="C117" s="9" t="s">
-        <v>278</v>
-      </c>
-      <c r="D117" s="10" t="s">
-        <v>279</v>
-      </c>
-      <c r="E117" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="F117" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="G117" s="10"/>
-      <c r="H117" s="10"/>
-      <c r="I117" s="9"/>
-    </row>
-    <row r="118" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A118" s="20" t="s">
-        <v>265</v>
-      </c>
-      <c r="B118" s="20"/>
-      <c r="C118" s="9" t="s">
-        <v>280</v>
-      </c>
-      <c r="D118" s="10" t="s">
-        <v>281</v>
-      </c>
-      <c r="E118" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="F118" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="G118" s="10"/>
-      <c r="H118" s="10"/>
-      <c r="I118" s="9"/>
-    </row>
-    <row r="119" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A119" s="21" t="s">
-        <v>282</v>
-      </c>
-      <c r="B119" s="21" t="s">
-        <v>283</v>
-      </c>
-      <c r="C119" s="9" t="s">
-        <v>284</v>
-      </c>
-      <c r="D119" s="10" t="s">
-        <v>285</v>
-      </c>
-      <c r="E119" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="F119" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="G119" s="10"/>
-      <c r="H119" s="10"/>
-      <c r="I119" s="9"/>
-    </row>
-    <row r="120" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A120" s="21" t="s">
-        <v>282</v>
-      </c>
-      <c r="B120" s="21" t="s">
-        <v>283</v>
-      </c>
-      <c r="C120" s="9" t="s">
-        <v>286</v>
-      </c>
-      <c r="D120" s="10" t="s">
-        <v>287</v>
-      </c>
-      <c r="E120" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="F120" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="G120" s="10"/>
-      <c r="H120" s="10"/>
-      <c r="I120" s="9"/>
-    </row>
-    <row r="121" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A121" s="21" t="s">
-        <v>282</v>
-      </c>
-      <c r="B121" s="21" t="s">
-        <v>288</v>
-      </c>
-      <c r="C121" s="9" t="s">
-        <v>289</v>
-      </c>
-      <c r="D121" s="10" t="s">
-        <v>290</v>
-      </c>
-      <c r="E121" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="F121" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="G121" s="10"/>
-      <c r="H121" s="10"/>
-      <c r="I121" s="9"/>
-    </row>
-    <row r="122" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A122" s="21" t="s">
-        <v>282</v>
-      </c>
-      <c r="B122" s="21" t="s">
-        <v>288</v>
-      </c>
-      <c r="C122" s="9" t="s">
-        <v>291</v>
-      </c>
-      <c r="D122" s="10" t="s">
-        <v>292</v>
-      </c>
-      <c r="E122" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="F122" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="G122" s="10"/>
-      <c r="H122" s="10"/>
-      <c r="I122" s="9"/>
-    </row>
-    <row r="123" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A123" s="21" t="s">
-        <v>282</v>
-      </c>
-      <c r="B123" s="21" t="s">
-        <v>288</v>
-      </c>
-      <c r="C123" s="9" t="s">
-        <v>293</v>
-      </c>
-      <c r="D123" s="10" t="s">
-        <v>294</v>
-      </c>
-      <c r="E123" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="F123" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="G123" s="10"/>
-      <c r="H123" s="10"/>
-      <c r="I123" s="9"/>
-    </row>
-    <row r="124" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A124" s="21" t="s">
-        <v>282</v>
-      </c>
-      <c r="B124" s="21" t="s">
-        <v>288</v>
-      </c>
-      <c r="C124" s="9" t="s">
-        <v>295</v>
-      </c>
-      <c r="D124" s="10" t="s">
-        <v>296</v>
-      </c>
-      <c r="E124" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="F124" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="G124" s="10"/>
-      <c r="H124" s="10"/>
-      <c r="I124" s="9"/>
-    </row>
-    <row r="125" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A125" s="21" t="s">
-        <v>282</v>
-      </c>
-      <c r="B125" s="21" t="s">
-        <v>288</v>
-      </c>
-      <c r="C125" s="9" t="s">
-        <v>297</v>
-      </c>
-      <c r="D125" s="10" t="s">
-        <v>298</v>
-      </c>
-      <c r="E125" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="F125" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="G125" s="10"/>
-      <c r="H125" s="10"/>
-      <c r="I125" s="9"/>
-    </row>
-    <row r="126" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A126" s="21" t="s">
-        <v>282</v>
-      </c>
-      <c r="B126" s="21" t="s">
-        <v>288</v>
-      </c>
-      <c r="C126" s="9" t="s">
-        <v>299</v>
-      </c>
-      <c r="D126" s="10" t="s">
-        <v>300</v>
-      </c>
-      <c r="E126" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="F126" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="G126" s="10"/>
-      <c r="H126" s="10"/>
-      <c r="I126" s="9"/>
-    </row>
-    <row r="127" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A127" s="21" t="s">
-        <v>282</v>
-      </c>
-      <c r="B127" s="21" t="s">
-        <v>288</v>
-      </c>
-      <c r="C127" s="9" t="s">
-        <v>301</v>
-      </c>
-      <c r="D127" s="10" t="s">
-        <v>302</v>
-      </c>
-      <c r="E127" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="F127" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="G127" s="10"/>
-      <c r="H127" s="10"/>
-      <c r="I127" s="9"/>
-    </row>
-    <row r="128" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A128" s="21" t="s">
-        <v>282</v>
-      </c>
-      <c r="B128" s="21" t="s">
-        <v>288</v>
-      </c>
-      <c r="C128" s="9" t="s">
-        <v>303</v>
-      </c>
-      <c r="D128" s="10" t="s">
-        <v>304</v>
-      </c>
-      <c r="E128" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="F128" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="G128" s="10"/>
-      <c r="H128" s="10"/>
-      <c r="I128" s="9"/>
-    </row>
-    <row r="129" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A129" s="21" t="s">
-        <v>282</v>
-      </c>
-      <c r="B129" s="21" t="s">
-        <v>305</v>
-      </c>
-      <c r="C129" s="9" t="s">
-        <v>306</v>
-      </c>
-      <c r="D129" s="10" t="s">
-        <v>307</v>
-      </c>
-      <c r="E129" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="F129" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="G129" s="10"/>
-      <c r="H129" s="10"/>
-      <c r="I129" s="9"/>
-    </row>
-    <row r="130" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A130" s="21" t="s">
-        <v>282</v>
-      </c>
-      <c r="B130" s="21" t="s">
-        <v>305</v>
-      </c>
-      <c r="C130" s="9" t="s">
-        <v>308</v>
-      </c>
-      <c r="D130" s="10" t="s">
-        <v>309</v>
-      </c>
-      <c r="E130" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="F130" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="G130" s="10"/>
-      <c r="H130" s="10"/>
-      <c r="I130" s="9"/>
-    </row>
-    <row r="131" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A131" s="21" t="s">
-        <v>282</v>
-      </c>
-      <c r="B131" s="21" t="s">
-        <v>305</v>
-      </c>
-      <c r="C131" s="9" t="s">
-        <v>310</v>
-      </c>
-      <c r="D131" s="10" t="s">
-        <v>311</v>
-      </c>
-      <c r="E131" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="F131" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="G131" s="10"/>
-      <c r="H131" s="10"/>
-      <c r="I131" s="9"/>
-    </row>
-    <row r="132" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A132" s="21" t="s">
-        <v>282</v>
-      </c>
-      <c r="B132" s="21" t="s">
-        <v>305</v>
-      </c>
-      <c r="C132" s="9" t="s">
-        <v>312</v>
-      </c>
-      <c r="D132" s="10" t="s">
-        <v>313</v>
-      </c>
-      <c r="E132" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="F132" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="G132" s="10"/>
-      <c r="H132" s="10"/>
-      <c r="I132" s="9"/>
-    </row>
-    <row r="133" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A133" s="21" t="s">
-        <v>282</v>
-      </c>
-      <c r="B133" s="21" t="s">
-        <v>305</v>
-      </c>
-      <c r="C133" s="9" t="s">
-        <v>314</v>
-      </c>
-      <c r="D133" s="10" t="s">
-        <v>315</v>
-      </c>
-      <c r="E133" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="F133" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="G133" s="10"/>
-      <c r="H133" s="10"/>
-      <c r="I133" s="9"/>
-    </row>
-    <row r="134" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A134" s="21" t="s">
-        <v>282</v>
-      </c>
-      <c r="B134" s="21" t="s">
-        <v>305</v>
-      </c>
-      <c r="C134" s="9" t="s">
-        <v>316</v>
-      </c>
-      <c r="D134" s="10" t="s">
-        <v>317</v>
-      </c>
-      <c r="E134" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="F134" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="G134" s="10"/>
-      <c r="H134" s="10"/>
-      <c r="I134" s="9"/>
-    </row>
-    <row r="135" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A135" s="21" t="s">
-        <v>282</v>
-      </c>
-      <c r="B135" s="21" t="s">
-        <v>318</v>
-      </c>
-      <c r="C135" s="9" t="s">
-        <v>319</v>
-      </c>
-      <c r="D135" s="10" t="s">
-        <v>320</v>
-      </c>
-      <c r="E135" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="F135" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="G135" s="10"/>
-      <c r="H135" s="10"/>
-      <c r="I135" s="9"/>
-    </row>
-    <row r="136" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A136" s="21" t="s">
-        <v>282</v>
-      </c>
-      <c r="B136" s="21" t="s">
-        <v>318</v>
-      </c>
-      <c r="C136" s="9" t="s">
-        <v>321</v>
-      </c>
-      <c r="D136" s="10" t="s">
-        <v>322</v>
-      </c>
-      <c r="E136" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="F136" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="G136" s="10"/>
-      <c r="H136" s="10"/>
-      <c r="I136" s="9"/>
-    </row>
-    <row r="137" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A137" s="21" t="s">
-        <v>282</v>
-      </c>
-      <c r="B137" s="21" t="s">
-        <v>323</v>
-      </c>
-      <c r="C137" s="9" t="s">
-        <v>324</v>
-      </c>
-      <c r="D137" s="10" t="s">
-        <v>325</v>
-      </c>
-      <c r="E137" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="F137" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="G137" s="10"/>
-      <c r="H137" s="10"/>
-      <c r="I137" s="9"/>
-    </row>
-    <row r="138" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A138" s="21" t="s">
-        <v>282</v>
-      </c>
-      <c r="B138" s="21" t="s">
-        <v>323</v>
-      </c>
-      <c r="C138" s="9" t="s">
-        <v>326</v>
-      </c>
-      <c r="D138" s="10" t="s">
-        <v>327</v>
-      </c>
-      <c r="E138" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="F138" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="G138" s="10"/>
-      <c r="H138" s="10"/>
-      <c r="I138" s="9"/>
-    </row>
-    <row r="139" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A139" s="21" t="s">
-        <v>282</v>
-      </c>
-      <c r="B139" s="21" t="s">
-        <v>323</v>
-      </c>
-      <c r="C139" s="9" t="s">
-        <v>328</v>
-      </c>
-      <c r="D139" s="10" t="s">
-        <v>329</v>
-      </c>
-      <c r="E139" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="F139" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="G139" s="10"/>
-      <c r="H139" s="10"/>
-      <c r="I139" s="9"/>
-    </row>
-    <row r="140" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A140" s="21" t="s">
-        <v>282</v>
-      </c>
-      <c r="B140" s="21" t="s">
-        <v>330</v>
-      </c>
-      <c r="C140" s="9" t="s">
-        <v>331</v>
-      </c>
-      <c r="D140" s="10" t="s">
-        <v>332</v>
-      </c>
-      <c r="E140" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="F140" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="G140" s="10"/>
-      <c r="H140" s="10"/>
-      <c r="I140" s="9"/>
-    </row>
-    <row r="141" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A141" s="21" t="s">
-        <v>282</v>
-      </c>
-      <c r="B141" s="21" t="s">
-        <v>330</v>
-      </c>
-      <c r="C141" s="9" t="s">
-        <v>333</v>
-      </c>
-      <c r="D141" s="10" t="s">
-        <v>334</v>
-      </c>
-      <c r="E141" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="F141" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="G141" s="10"/>
-      <c r="H141" s="10"/>
-      <c r="I141" s="9"/>
-    </row>
-    <row r="142" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A142" s="21" t="s">
-        <v>282</v>
-      </c>
-      <c r="B142" s="21" t="s">
-        <v>330</v>
-      </c>
-      <c r="C142" s="9" t="s">
-        <v>335</v>
-      </c>
-      <c r="D142" s="10" t="s">
-        <v>336</v>
-      </c>
-      <c r="E142" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="F142" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="G142" s="10"/>
-      <c r="H142" s="10"/>
-      <c r="I142" s="9"/>
-    </row>
-    <row r="143" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A143" s="21" t="s">
-        <v>282</v>
-      </c>
-      <c r="B143" s="21" t="s">
-        <v>337</v>
-      </c>
-      <c r="C143" s="9" t="s">
-        <v>338</v>
-      </c>
-      <c r="D143" s="10" t="s">
-        <v>339</v>
-      </c>
-      <c r="E143" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="F143" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="G143" s="10"/>
-      <c r="H143" s="10"/>
-      <c r="I143" s="9"/>
-    </row>
-    <row r="144" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A144" s="21" t="s">
-        <v>282</v>
-      </c>
-      <c r="B144" s="21" t="s">
-        <v>337</v>
-      </c>
-      <c r="C144" s="9" t="s">
-        <v>340</v>
-      </c>
-      <c r="D144" s="10" t="s">
-        <v>341</v>
-      </c>
-      <c r="E144" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="F144" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="G144" s="10"/>
-      <c r="H144" s="10"/>
-      <c r="I144" s="9"/>
-    </row>
-    <row r="145" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A145" s="21" t="s">
-        <v>282</v>
-      </c>
-      <c r="B145" s="21" t="s">
-        <v>337</v>
-      </c>
-      <c r="C145" s="9" t="s">
-        <v>342</v>
-      </c>
-      <c r="D145" s="10" t="s">
-        <v>343</v>
-      </c>
-      <c r="E145" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="F145" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="G145" s="10"/>
-      <c r="H145" s="10"/>
-      <c r="I145" s="9"/>
-    </row>
-    <row r="146" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A146" s="21" t="s">
-        <v>282</v>
-      </c>
-      <c r="B146" s="21" t="s">
-        <v>337</v>
-      </c>
-      <c r="C146" s="9" t="s">
-        <v>344</v>
-      </c>
-      <c r="D146" s="10" t="s">
-        <v>345</v>
-      </c>
-      <c r="E146" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="F146" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="G146" s="10"/>
-      <c r="H146" s="10"/>
-      <c r="I146" s="9"/>
-    </row>
-    <row r="147" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A147" s="21" t="s">
-        <v>282</v>
-      </c>
-      <c r="B147" s="21" t="s">
-        <v>337</v>
-      </c>
-      <c r="C147" s="9" t="s">
-        <v>346</v>
-      </c>
-      <c r="D147" s="10" t="s">
-        <v>347</v>
-      </c>
-      <c r="E147" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="F147" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="G147" s="10"/>
-      <c r="H147" s="10"/>
-      <c r="I147" s="9"/>
-    </row>
-    <row r="148" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A148" s="21" t="s">
-        <v>282</v>
-      </c>
-      <c r="B148" s="21" t="s">
-        <v>337</v>
-      </c>
-      <c r="C148" s="9" t="s">
-        <v>348</v>
-      </c>
-      <c r="D148" s="10" t="s">
-        <v>349</v>
-      </c>
-      <c r="E148" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="F148" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="G148" s="10"/>
-      <c r="H148" s="10"/>
-      <c r="I148" s="9"/>
-    </row>
-    <row r="149" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A149" s="21" t="s">
-        <v>282</v>
-      </c>
-      <c r="B149" s="21" t="s">
-        <v>350</v>
-      </c>
-      <c r="C149" s="9" t="s">
-        <v>351</v>
-      </c>
-      <c r="D149" s="10" t="s">
-        <v>352</v>
-      </c>
-      <c r="E149" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="F149" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="G149" s="10"/>
-      <c r="H149" s="10"/>
-      <c r="I149" s="9"/>
-    </row>
-    <row r="150" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A150" s="21" t="s">
-        <v>282</v>
-      </c>
-      <c r="B150" s="21" t="s">
-        <v>350</v>
-      </c>
-      <c r="C150" s="9" t="s">
-        <v>353</v>
-      </c>
-      <c r="D150" s="10" t="s">
-        <v>354</v>
-      </c>
-      <c r="E150" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="F150" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="G150" s="10"/>
-      <c r="H150" s="10"/>
-      <c r="I150" s="9"/>
-    </row>
-    <row r="151" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A151" s="21" t="s">
-        <v>282</v>
-      </c>
-      <c r="B151" s="21" t="s">
-        <v>350</v>
-      </c>
-      <c r="C151" s="9" t="s">
-        <v>355</v>
-      </c>
-      <c r="D151" s="10" t="s">
-        <v>356</v>
-      </c>
-      <c r="E151" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="F151" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="G151" s="10"/>
-      <c r="H151" s="10"/>
-      <c r="I151" s="9"/>
-    </row>
-    <row r="152" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A152" s="21" t="s">
-        <v>282</v>
-      </c>
-      <c r="B152" s="21" t="s">
-        <v>350</v>
-      </c>
-      <c r="C152" s="9" t="s">
-        <v>357</v>
-      </c>
-      <c r="D152" s="10" t="s">
-        <v>358</v>
-      </c>
-      <c r="E152" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="F152" s="10" t="s">
-        <v>359</v>
-      </c>
-      <c r="G152" s="10"/>
-      <c r="H152" s="10"/>
-      <c r="I152" s="9"/>
-    </row>
-    <row r="153" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A153" s="21" t="s">
-        <v>282</v>
-      </c>
-      <c r="B153" s="21" t="s">
-        <v>360</v>
-      </c>
-      <c r="C153" s="9" t="s">
-        <v>361</v>
-      </c>
-      <c r="D153" s="10" t="s">
-        <v>362</v>
-      </c>
-      <c r="E153" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="F153" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="G153" s="10"/>
-      <c r="H153" s="10"/>
-      <c r="I153" s="9"/>
-    </row>
-    <row r="154" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A154" s="21" t="s">
-        <v>282</v>
-      </c>
-      <c r="B154" s="21" t="s">
-        <v>360</v>
-      </c>
-      <c r="C154" s="9" t="s">
-        <v>363</v>
-      </c>
-      <c r="D154" s="10" t="s">
-        <v>364</v>
-      </c>
-      <c r="E154" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="F154" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="G154" s="10"/>
-      <c r="H154" s="10"/>
-      <c r="I154" s="9"/>
-    </row>
-    <row r="155" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A155" s="21" t="s">
-        <v>282</v>
-      </c>
-      <c r="B155" s="21" t="s">
-        <v>365</v>
-      </c>
-      <c r="C155" s="9" t="s">
-        <v>366</v>
-      </c>
-      <c r="D155" s="10" t="s">
-        <v>367</v>
-      </c>
-      <c r="E155" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="F155" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="G155" s="10"/>
-      <c r="H155" s="10"/>
-      <c r="I155" s="9"/>
-    </row>
-    <row r="156" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A156" s="21" t="s">
-        <v>282</v>
-      </c>
-      <c r="B156" s="21" t="s">
-        <v>365</v>
-      </c>
-      <c r="C156" s="9" t="s">
-        <v>368</v>
-      </c>
-      <c r="D156" s="10" t="s">
-        <v>369</v>
-      </c>
-      <c r="E156" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="F156" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="G156" s="10"/>
-      <c r="H156" s="10"/>
-      <c r="I156" s="9"/>
-    </row>
-    <row r="157" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A157" s="21" t="s">
-        <v>282</v>
-      </c>
-      <c r="B157" s="21" t="s">
-        <v>365</v>
-      </c>
-      <c r="C157" s="9" t="s">
-        <v>370</v>
-      </c>
-      <c r="D157" s="10" t="s">
-        <v>371</v>
-      </c>
-      <c r="E157" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="F157" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="G157" s="10"/>
-      <c r="H157" s="10"/>
-      <c r="I157" s="9"/>
-    </row>
-    <row r="158" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A158" s="21" t="s">
-        <v>282</v>
-      </c>
-      <c r="B158" s="21" t="s">
-        <v>372</v>
-      </c>
-      <c r="C158" s="9" t="s">
-        <v>373</v>
-      </c>
-      <c r="D158" s="10" t="s">
-        <v>374</v>
-      </c>
-      <c r="E158" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="F158" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="G158" s="10"/>
-      <c r="H158" s="10"/>
-      <c r="I158" s="9"/>
-    </row>
-    <row r="159" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A159" s="21" t="s">
-        <v>282</v>
-      </c>
-      <c r="B159" s="21" t="s">
-        <v>372</v>
-      </c>
-      <c r="C159" s="9" t="s">
-        <v>375</v>
-      </c>
-      <c r="D159" s="10" t="s">
-        <v>376</v>
-      </c>
-      <c r="E159" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="F159" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="G159" s="10"/>
-      <c r="H159" s="10"/>
-      <c r="I159" s="9"/>
-    </row>
-    <row r="160" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A160" s="21" t="s">
-        <v>282</v>
-      </c>
-      <c r="B160" s="21" t="s">
-        <v>372</v>
-      </c>
-      <c r="C160" s="9" t="s">
-        <v>377</v>
-      </c>
-      <c r="D160" s="10" t="s">
-        <v>378</v>
-      </c>
-      <c r="E160" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="F160" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="G160" s="10"/>
-      <c r="H160" s="10"/>
-      <c r="I160" s="9"/>
-    </row>
-    <row r="161" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A161" s="21" t="s">
-        <v>282</v>
-      </c>
-      <c r="B161" s="21" t="s">
-        <v>372</v>
-      </c>
-      <c r="C161" s="9" t="s">
-        <v>379</v>
-      </c>
-      <c r="D161" s="10" t="s">
-        <v>380</v>
-      </c>
-      <c r="E161" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="F161" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="G161" s="10"/>
-      <c r="H161" s="10"/>
-      <c r="I161" s="9"/>
-    </row>
-    <row r="162" customFormat="false" ht="35.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A162" s="21" t="s">
-        <v>282</v>
-      </c>
-      <c r="B162" s="21"/>
-      <c r="C162" s="9" t="s">
-        <v>381</v>
-      </c>
-      <c r="D162" s="10" t="s">
-        <v>382</v>
-      </c>
-      <c r="E162" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="F162" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="G162" s="10"/>
-      <c r="H162" s="10"/>
-      <c r="I162" s="9" t="s">
-        <v>383</v>
-      </c>
-    </row>
-    <row r="163" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A163" s="21" t="s">
-        <v>282</v>
-      </c>
-      <c r="B163" s="21"/>
-      <c r="C163" s="9" t="s">
-        <v>384</v>
-      </c>
-      <c r="D163" s="10" t="s">
-        <v>385</v>
-      </c>
-      <c r="E163" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="F163" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="G163" s="10"/>
-      <c r="H163" s="10"/>
-      <c r="I163" s="9" t="s">
-        <v>386</v>
-      </c>
-    </row>
-    <row r="164" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A164" s="21" t="s">
-        <v>282</v>
-      </c>
-      <c r="B164" s="21"/>
-      <c r="C164" s="9" t="s">
-        <v>387</v>
-      </c>
-      <c r="D164" s="10" t="s">
-        <v>388</v>
-      </c>
-      <c r="E164" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="F164" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="G164" s="10"/>
-      <c r="H164" s="10"/>
-      <c r="I164" s="9"/>
-    </row>
-    <row r="165" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A165" s="21" t="s">
-        <v>282</v>
-      </c>
-      <c r="B165" s="21"/>
-      <c r="C165" s="9" t="s">
-        <v>389</v>
-      </c>
-      <c r="D165" s="10" t="s">
-        <v>390</v>
-      </c>
-      <c r="E165" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="F165" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="G165" s="10"/>
-      <c r="H165" s="10"/>
-      <c r="I165" s="9" t="s">
-        <v>391</v>
-      </c>
-    </row>
-    <row r="166" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A166" s="21" t="s">
-        <v>282</v>
-      </c>
-      <c r="B166" s="21"/>
-      <c r="C166" s="9" t="s">
-        <v>392</v>
-      </c>
-      <c r="D166" s="10" t="s">
-        <v>393</v>
-      </c>
-      <c r="E166" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="F166" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="G166" s="10"/>
-      <c r="H166" s="10"/>
-      <c r="I166" s="9" t="s">
-        <v>394</v>
-      </c>
-    </row>
-    <row r="167" customFormat="false" ht="35.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A167" s="21" t="s">
-        <v>282</v>
-      </c>
-      <c r="B167" s="21"/>
-      <c r="C167" s="9" t="s">
-        <v>395</v>
-      </c>
-      <c r="D167" s="10" t="s">
-        <v>396</v>
-      </c>
-      <c r="E167" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="F167" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="G167" s="10"/>
-      <c r="H167" s="10"/>
-      <c r="I167" s="9" t="s">
-        <v>397</v>
-      </c>
-    </row>
-    <row r="168" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A168" s="21" t="s">
-        <v>282</v>
-      </c>
-      <c r="B168" s="21"/>
-      <c r="C168" s="9" t="s">
-        <v>398</v>
-      </c>
-      <c r="D168" s="10" t="s">
-        <v>399</v>
-      </c>
-      <c r="E168" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="F168" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="G168" s="10"/>
-      <c r="H168" s="10"/>
-      <c r="I168" s="9" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="169" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A169" s="22" t="s">
-        <v>401</v>
-      </c>
-      <c r="B169" s="22"/>
-      <c r="C169" s="9" t="s">
-        <v>402</v>
-      </c>
-      <c r="D169" s="10" t="s">
-        <v>403</v>
-      </c>
-      <c r="E169" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="F169" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="G169" s="10"/>
-      <c r="H169" s="10"/>
-      <c r="I169" s="9"/>
-    </row>
-    <row r="170" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A170" s="22" t="s">
-        <v>401</v>
-      </c>
-      <c r="B170" s="22"/>
-      <c r="C170" s="9" t="s">
-        <v>404</v>
-      </c>
-      <c r="D170" s="10" t="s">
-        <v>405</v>
-      </c>
-      <c r="E170" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="F170" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="G170" s="10"/>
-      <c r="H170" s="10"/>
-      <c r="I170" s="9"/>
-    </row>
-    <row r="171" customFormat="false" ht="52.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A171" s="23" t="s">
-        <v>406</v>
-      </c>
-      <c r="B171" s="23"/>
-      <c r="C171" s="9" t="s">
-        <v>407</v>
-      </c>
-      <c r="D171" s="10" t="s">
-        <v>408</v>
-      </c>
-      <c r="E171" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="F171" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="G171" s="10"/>
-      <c r="H171" s="10"/>
-      <c r="I171" s="9"/>
-    </row>
-    <row r="172" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A172" s="23" t="s">
-        <v>406</v>
-      </c>
-      <c r="B172" s="23"/>
-      <c r="C172" s="9" t="s">
-        <v>409</v>
-      </c>
-      <c r="D172" s="10" t="s">
-        <v>410</v>
-      </c>
-      <c r="E172" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="F172" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="G172" s="10"/>
-      <c r="H172" s="10"/>
-      <c r="I172" s="9"/>
-    </row>
-    <row r="173" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A173" s="23" t="s">
-        <v>406</v>
-      </c>
-      <c r="B173" s="23"/>
-      <c r="C173" s="9"/>
-      <c r="D173" s="10" t="s">
-        <v>411</v>
-      </c>
-      <c r="E173" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="F173" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="G173" s="10"/>
-      <c r="H173" s="10"/>
-      <c r="I173" s="9"/>
-    </row>
-    <row r="174" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A174" s="23" t="s">
-        <v>406</v>
-      </c>
-      <c r="B174" s="23"/>
-      <c r="C174" s="9"/>
-      <c r="D174" s="10" t="s">
-        <v>412</v>
-      </c>
-      <c r="E174" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="F174" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="G174" s="10"/>
-      <c r="H174" s="10"/>
-      <c r="I174" s="9"/>
-    </row>
-    <row r="175" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A175" s="23" t="s">
-        <v>406</v>
-      </c>
-      <c r="B175" s="23"/>
-      <c r="C175" s="9" t="s">
-        <v>413</v>
-      </c>
-      <c r="D175" s="10" t="s">
-        <v>414</v>
-      </c>
-      <c r="E175" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="F175" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="G175" s="10"/>
-      <c r="H175" s="10"/>
-      <c r="I175" s="9"/>
-    </row>
-    <row r="176" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A176" s="23" t="s">
-        <v>406</v>
-      </c>
-      <c r="B176" s="23"/>
-      <c r="C176" s="9" t="s">
-        <v>415</v>
-      </c>
-      <c r="D176" s="10" t="s">
-        <v>416</v>
-      </c>
-      <c r="E176" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="F176" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="G176" s="10"/>
-      <c r="H176" s="10"/>
-      <c r="I176" s="9"/>
-    </row>
-    <row r="177" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A177" s="23" t="s">
-        <v>406</v>
-      </c>
-      <c r="B177" s="23"/>
-      <c r="C177" s="9" t="s">
-        <v>417</v>
-      </c>
-      <c r="D177" s="10" t="s">
-        <v>418</v>
-      </c>
-      <c r="E177" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="F177" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="G177" s="10"/>
-      <c r="H177" s="10"/>
-      <c r="I177" s="9"/>
-    </row>
-    <row r="178" customFormat="false" ht="46.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A178" s="24" t="s">
-        <v>419</v>
-      </c>
-      <c r="B178" s="23" t="s">
-        <v>420</v>
-      </c>
-      <c r="C178" s="9" t="s">
-        <v>421</v>
-      </c>
-      <c r="D178" s="10" t="s">
-        <v>422</v>
-      </c>
-      <c r="E178" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="F178" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="G178" s="10"/>
-      <c r="H178" s="10"/>
-      <c r="I178" s="9" t="s">
-        <v>423</v>
-      </c>
-    </row>
-    <row r="179" customFormat="false" ht="35.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A179" s="24" t="s">
-        <v>419</v>
-      </c>
-      <c r="B179" s="23" t="s">
-        <v>424</v>
-      </c>
-      <c r="C179" s="9" t="s">
-        <v>425</v>
-      </c>
-      <c r="D179" s="10" t="s">
-        <v>426</v>
-      </c>
-      <c r="E179" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="F179" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="G179" s="10"/>
-      <c r="H179" s="10"/>
-      <c r="I179" s="9" t="s">
+      <c r="I116" s="9" t="s">
         <v>427</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I179"/>
+  <autoFilter ref="A1:I116"/>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E2:F179" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E2:F116" type="list">
       <formula1>"À tester,Oui,Non,Partiel"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -6259,23 +4936,23 @@
         <v>20</v>
       </c>
       <c r="B4" s="27" t="n">
-        <f aca="false">COUNTIF(Blocs!$A$2:$A$179,A4)</f>
+        <f aca="false">COUNTIF(Blocs!$A$2:$A$116,A4)</f>
         <v>5</v>
       </c>
       <c r="C4" s="27" t="n">
-        <f aca="false">COUNTIFS(Blocs!$A$2:$A$179,A4,Blocs!$E$2:$E$179,"&lt;&gt;À tester")</f>
+        <f aca="false">COUNTIFS(Blocs!$A$2:$A$116,A4,Blocs!$E$2:$E$116,"&lt;&gt;À tester")</f>
         <v>3</v>
       </c>
       <c r="D4" s="27" t="n">
-        <f aca="false">COUNTIFS(Blocs!$A$2:$A$179,A4,Blocs!$E$2:$E$179,"Oui")</f>
+        <f aca="false">COUNTIFS(Blocs!$A$2:$A$116,A4,Blocs!$E$2:$E$116,"Oui")</f>
         <v>2</v>
       </c>
       <c r="E4" s="27" t="n">
-        <f aca="false">COUNTIFS(Blocs!$A$2:$A$179,A4,Blocs!$F$2:$F$179,"&lt;&gt;À tester")</f>
+        <f aca="false">COUNTIFS(Blocs!$A$2:$A$116,A4,Blocs!$F$2:$F$116,"&lt;&gt;À tester")</f>
         <v>5</v>
       </c>
       <c r="F4" s="27" t="n">
-        <f aca="false">COUNTIFS(Blocs!$A$2:$A$179,A4,Blocs!$F$2:$F$179,"Oui")</f>
+        <f aca="false">COUNTIFS(Blocs!$A$2:$A$116,A4,Blocs!$F$2:$F$116,"Oui")</f>
         <v>5</v>
       </c>
     </row>
@@ -6284,23 +4961,23 @@
         <v>41</v>
       </c>
       <c r="B5" s="27" t="n">
-        <f aca="false">COUNTIF(Blocs!$A$2:$A$179,A5)</f>
+        <f aca="false">COUNTIF(Blocs!$A$2:$A$116,A5)</f>
         <v>5</v>
       </c>
       <c r="C5" s="27" t="n">
-        <f aca="false">COUNTIFS(Blocs!$A$2:$A$179,A5,Blocs!$E$2:$E$179,"&lt;&gt;À tester")</f>
+        <f aca="false">COUNTIFS(Blocs!$A$2:$A$116,A5,Blocs!$E$2:$E$116,"&lt;&gt;À tester")</f>
         <v>5</v>
       </c>
       <c r="D5" s="27" t="n">
-        <f aca="false">COUNTIFS(Blocs!$A$2:$A$179,A5,Blocs!$E$2:$E$179,"Oui")</f>
+        <f aca="false">COUNTIFS(Blocs!$A$2:$A$116,A5,Blocs!$E$2:$E$116,"Oui")</f>
         <v>5</v>
       </c>
       <c r="E5" s="27" t="n">
-        <f aca="false">COUNTIFS(Blocs!$A$2:$A$179,A5,Blocs!$F$2:$F$179,"&lt;&gt;À tester")</f>
+        <f aca="false">COUNTIFS(Blocs!$A$2:$A$116,A5,Blocs!$F$2:$F$116,"&lt;&gt;À tester")</f>
         <v>5</v>
       </c>
       <c r="F5" s="27" t="n">
-        <f aca="false">COUNTIFS(Blocs!$A$2:$A$179,A5,Blocs!$F$2:$F$179,"Oui")</f>
+        <f aca="false">COUNTIFS(Blocs!$A$2:$A$116,A5,Blocs!$F$2:$F$116,"Oui")</f>
         <v>5</v>
       </c>
     </row>
@@ -6309,23 +4986,23 @@
         <v>52</v>
       </c>
       <c r="B6" s="27" t="n">
-        <f aca="false">COUNTIF(Blocs!$A$2:$A$179,A6)</f>
+        <f aca="false">COUNTIF(Blocs!$A$2:$A$116,A6)</f>
         <v>7</v>
       </c>
       <c r="C6" s="27" t="n">
-        <f aca="false">COUNTIFS(Blocs!$A$2:$A$179,A6,Blocs!$E$2:$E$179,"&lt;&gt;À tester")</f>
+        <f aca="false">COUNTIFS(Blocs!$A$2:$A$116,A6,Blocs!$E$2:$E$116,"&lt;&gt;À tester")</f>
         <v>6</v>
       </c>
       <c r="D6" s="27" t="n">
-        <f aca="false">COUNTIFS(Blocs!$A$2:$A$179,A6,Blocs!$E$2:$E$179,"Oui")</f>
+        <f aca="false">COUNTIFS(Blocs!$A$2:$A$116,A6,Blocs!$E$2:$E$116,"Oui")</f>
         <v>6</v>
       </c>
       <c r="E6" s="27" t="n">
-        <f aca="false">COUNTIFS(Blocs!$A$2:$A$179,A6,Blocs!$F$2:$F$179,"&lt;&gt;À tester")</f>
+        <f aca="false">COUNTIFS(Blocs!$A$2:$A$116,A6,Blocs!$F$2:$F$116,"&lt;&gt;À tester")</f>
         <v>6</v>
       </c>
       <c r="F6" s="27" t="n">
-        <f aca="false">COUNTIFS(Blocs!$A$2:$A$179,A6,Blocs!$F$2:$F$179,"Oui")</f>
+        <f aca="false">COUNTIFS(Blocs!$A$2:$A$116,A6,Blocs!$F$2:$F$116,"Oui")</f>
         <v>6</v>
       </c>
     </row>
@@ -6334,23 +5011,23 @@
         <v>68</v>
       </c>
       <c r="B7" s="27" t="n">
-        <f aca="false">COUNTIF(Blocs!$A$2:$A$179,A7)</f>
+        <f aca="false">COUNTIF(Blocs!$A$2:$A$116,A7)</f>
         <v>18</v>
       </c>
       <c r="C7" s="27" t="n">
-        <f aca="false">COUNTIFS(Blocs!$A$2:$A$179,A7,Blocs!$E$2:$E$179,"&lt;&gt;À tester")</f>
+        <f aca="false">COUNTIFS(Blocs!$A$2:$A$116,A7,Blocs!$E$2:$E$116,"&lt;&gt;À tester")</f>
         <v>0</v>
       </c>
       <c r="D7" s="27" t="n">
-        <f aca="false">COUNTIFS(Blocs!$A$2:$A$179,A7,Blocs!$E$2:$E$179,"Oui")</f>
+        <f aca="false">COUNTIFS(Blocs!$A$2:$A$116,A7,Blocs!$E$2:$E$116,"Oui")</f>
         <v>0</v>
       </c>
       <c r="E7" s="27" t="n">
-        <f aca="false">COUNTIFS(Blocs!$A$2:$A$179,A7,Blocs!$F$2:$F$179,"&lt;&gt;À tester")</f>
+        <f aca="false">COUNTIFS(Blocs!$A$2:$A$116,A7,Blocs!$F$2:$F$116,"&lt;&gt;À tester")</f>
         <v>0</v>
       </c>
       <c r="F7" s="27" t="n">
-        <f aca="false">COUNTIFS(Blocs!$A$2:$A$179,A7,Blocs!$F$2:$F$179,"Oui")</f>
+        <f aca="false">COUNTIFS(Blocs!$A$2:$A$116,A7,Blocs!$F$2:$F$116,"Oui")</f>
         <v>0</v>
       </c>
     </row>
@@ -6359,23 +5036,23 @@
         <v>107</v>
       </c>
       <c r="B8" s="27" t="n">
-        <f aca="false">COUNTIF(Blocs!$A$2:$A$179,A8)</f>
+        <f aca="false">COUNTIF(Blocs!$A$2:$A$116,A8)</f>
         <v>4</v>
       </c>
       <c r="C8" s="27" t="n">
-        <f aca="false">COUNTIFS(Blocs!$A$2:$A$179,A8,Blocs!$E$2:$E$179,"&lt;&gt;À tester")</f>
+        <f aca="false">COUNTIFS(Blocs!$A$2:$A$116,A8,Blocs!$E$2:$E$116,"&lt;&gt;À tester")</f>
         <v>0</v>
       </c>
       <c r="D8" s="27" t="n">
-        <f aca="false">COUNTIFS(Blocs!$A$2:$A$179,A8,Blocs!$E$2:$E$179,"Oui")</f>
+        <f aca="false">COUNTIFS(Blocs!$A$2:$A$116,A8,Blocs!$E$2:$E$116,"Oui")</f>
         <v>0</v>
       </c>
       <c r="E8" s="27" t="n">
-        <f aca="false">COUNTIFS(Blocs!$A$2:$A$179,A8,Blocs!$F$2:$F$179,"&lt;&gt;À tester")</f>
+        <f aca="false">COUNTIFS(Blocs!$A$2:$A$116,A8,Blocs!$F$2:$F$116,"&lt;&gt;À tester")</f>
         <v>0</v>
       </c>
       <c r="F8" s="27" t="n">
-        <f aca="false">COUNTIFS(Blocs!$A$2:$A$179,A8,Blocs!$F$2:$F$179,"Oui")</f>
+        <f aca="false">COUNTIFS(Blocs!$A$2:$A$116,A8,Blocs!$F$2:$F$116,"Oui")</f>
         <v>0</v>
       </c>
     </row>
@@ -6384,23 +5061,23 @@
         <v>116</v>
       </c>
       <c r="B9" s="27" t="n">
-        <f aca="false">COUNTIF(Blocs!$A$2:$A$179,A9)</f>
+        <f aca="false">COUNTIF(Blocs!$A$2:$A$116,A9)</f>
         <v>9</v>
       </c>
       <c r="C9" s="27" t="n">
-        <f aca="false">COUNTIFS(Blocs!$A$2:$A$179,A9,Blocs!$E$2:$E$179,"&lt;&gt;À tester")</f>
+        <f aca="false">COUNTIFS(Blocs!$A$2:$A$116,A9,Blocs!$E$2:$E$116,"&lt;&gt;À tester")</f>
         <v>0</v>
       </c>
       <c r="D9" s="27" t="n">
-        <f aca="false">COUNTIFS(Blocs!$A$2:$A$179,A9,Blocs!$E$2:$E$179,"Oui")</f>
+        <f aca="false">COUNTIFS(Blocs!$A$2:$A$116,A9,Blocs!$E$2:$E$116,"Oui")</f>
         <v>0</v>
       </c>
       <c r="E9" s="27" t="n">
-        <f aca="false">COUNTIFS(Blocs!$A$2:$A$179,A9,Blocs!$F$2:$F$179,"&lt;&gt;À tester")</f>
+        <f aca="false">COUNTIFS(Blocs!$A$2:$A$116,A9,Blocs!$F$2:$F$116,"&lt;&gt;À tester")</f>
         <v>0</v>
       </c>
       <c r="F9" s="27" t="n">
-        <f aca="false">COUNTIFS(Blocs!$A$2:$A$179,A9,Blocs!$F$2:$F$179,"Oui")</f>
+        <f aca="false">COUNTIFS(Blocs!$A$2:$A$116,A9,Blocs!$F$2:$F$116,"Oui")</f>
         <v>0</v>
       </c>
     </row>
@@ -6409,248 +5086,148 @@
         <v>139</v>
       </c>
       <c r="B10" s="27" t="n">
-        <f aca="false">COUNTIF(Blocs!$A$2:$A$179,A10)</f>
+        <f aca="false">COUNTIF(Blocs!$A$2:$A$116,A10)</f>
         <v>6</v>
       </c>
       <c r="C10" s="27" t="n">
-        <f aca="false">COUNTIFS(Blocs!$A$2:$A$179,A10,Blocs!$E$2:$E$179,"&lt;&gt;À tester")</f>
+        <f aca="false">COUNTIFS(Blocs!$A$2:$A$116,A10,Blocs!$E$2:$E$116,"&lt;&gt;À tester")</f>
         <v>0</v>
       </c>
       <c r="D10" s="27" t="n">
-        <f aca="false">COUNTIFS(Blocs!$A$2:$A$179,A10,Blocs!$E$2:$E$179,"Oui")</f>
+        <f aca="false">COUNTIFS(Blocs!$A$2:$A$116,A10,Blocs!$E$2:$E$116,"Oui")</f>
         <v>0</v>
       </c>
       <c r="E10" s="27" t="n">
-        <f aca="false">COUNTIFS(Blocs!$A$2:$A$179,A10,Blocs!$F$2:$F$179,"&lt;&gt;À tester")</f>
+        <f aca="false">COUNTIFS(Blocs!$A$2:$A$116,A10,Blocs!$F$2:$F$116,"&lt;&gt;À tester")</f>
         <v>0</v>
       </c>
       <c r="F10" s="27" t="n">
-        <f aca="false">COUNTIFS(Blocs!$A$2:$A$179,A10,Blocs!$F$2:$F$179,"Oui")</f>
+        <f aca="false">COUNTIFS(Blocs!$A$2:$A$116,A10,Blocs!$F$2:$F$116,"Oui")</f>
         <v>0</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="26" t="s">
-        <v>152</v>
+        <v>282</v>
       </c>
       <c r="B11" s="27" t="n">
-        <f aca="false">COUNTIF(Blocs!$A$2:$A$179,A11)</f>
-        <v>27</v>
+        <f aca="false">COUNTIF(Blocs!$A$2:$A$116,A11)</f>
+        <v>50</v>
       </c>
       <c r="C11" s="27" t="n">
-        <f aca="false">COUNTIFS(Blocs!$A$2:$A$179,A11,Blocs!$E$2:$E$179,"&lt;&gt;À tester")</f>
-        <v>0</v>
+        <f aca="false">COUNTIFS(Blocs!$A$2:$A$116,A11,Blocs!$E$2:$E$116,"&lt;&gt;À tester")</f>
+        <v>4</v>
       </c>
       <c r="D11" s="27" t="n">
-        <f aca="false">COUNTIFS(Blocs!$A$2:$A$179,A11,Blocs!$E$2:$E$179,"Oui")</f>
-        <v>0</v>
+        <f aca="false">COUNTIFS(Blocs!$A$2:$A$116,A11,Blocs!$E$2:$E$116,"Oui")</f>
+        <v>4</v>
       </c>
       <c r="E11" s="27" t="n">
-        <f aca="false">COUNTIFS(Blocs!$A$2:$A$179,A11,Blocs!$F$2:$F$179,"&lt;&gt;À tester")</f>
-        <v>0</v>
+        <f aca="false">COUNTIFS(Blocs!$A$2:$A$116,A11,Blocs!$F$2:$F$116,"&lt;&gt;À tester")</f>
+        <v>4</v>
       </c>
       <c r="F11" s="27" t="n">
-        <f aca="false">COUNTIFS(Blocs!$A$2:$A$179,A11,Blocs!$F$2:$F$179,"Oui")</f>
-        <v>0</v>
+        <f aca="false">COUNTIFS(Blocs!$A$2:$A$116,A11,Blocs!$F$2:$F$116,"Oui")</f>
+        <v>3</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="26" t="s">
-        <v>207</v>
+        <v>401</v>
       </c>
       <c r="B12" s="27" t="n">
-        <f aca="false">COUNTIF(Blocs!$A$2:$A$179,A12)</f>
-        <v>7</v>
+        <f aca="false">COUNTIF(Blocs!$A$2:$A$116,A12)</f>
+        <v>2</v>
       </c>
       <c r="C12" s="27" t="n">
-        <f aca="false">COUNTIFS(Blocs!$A$2:$A$179,A12,Blocs!$E$2:$E$179,"&lt;&gt;À tester")</f>
+        <f aca="false">COUNTIFS(Blocs!$A$2:$A$116,A12,Blocs!$E$2:$E$116,"&lt;&gt;À tester")</f>
         <v>0</v>
       </c>
       <c r="D12" s="27" t="n">
-        <f aca="false">COUNTIFS(Blocs!$A$2:$A$179,A12,Blocs!$E$2:$E$179,"Oui")</f>
+        <f aca="false">COUNTIFS(Blocs!$A$2:$A$116,A12,Blocs!$E$2:$E$116,"Oui")</f>
         <v>0</v>
       </c>
       <c r="E12" s="27" t="n">
-        <f aca="false">COUNTIFS(Blocs!$A$2:$A$179,A12,Blocs!$F$2:$F$179,"&lt;&gt;À tester")</f>
+        <f aca="false">COUNTIFS(Blocs!$A$2:$A$116,A12,Blocs!$F$2:$F$116,"&lt;&gt;À tester")</f>
         <v>0</v>
       </c>
       <c r="F12" s="27" t="n">
-        <f aca="false">COUNTIFS(Blocs!$A$2:$A$179,A12,Blocs!$F$2:$F$179,"Oui")</f>
+        <f aca="false">COUNTIFS(Blocs!$A$2:$A$116,A12,Blocs!$F$2:$F$116,"Oui")</f>
         <v>0</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="26" t="s">
-        <v>222</v>
+        <v>406</v>
       </c>
       <c r="B13" s="27" t="n">
-        <f aca="false">COUNTIF(Blocs!$A$2:$A$179,A13)</f>
-        <v>21</v>
+        <f aca="false">COUNTIF(Blocs!$A$2:$A$116,A13)</f>
+        <v>7</v>
       </c>
       <c r="C13" s="27" t="n">
-        <f aca="false">COUNTIFS(Blocs!$A$2:$A$179,A13,Blocs!$E$2:$E$179,"&lt;&gt;À tester")</f>
-        <v>0</v>
+        <f aca="false">COUNTIFS(Blocs!$A$2:$A$116,A13,Blocs!$E$2:$E$116,"&lt;&gt;À tester")</f>
+        <v>1</v>
       </c>
       <c r="D13" s="27" t="n">
-        <f aca="false">COUNTIFS(Blocs!$A$2:$A$179,A13,Blocs!$E$2:$E$179,"Oui")</f>
-        <v>0</v>
+        <f aca="false">COUNTIFS(Blocs!$A$2:$A$116,A13,Blocs!$E$2:$E$116,"Oui")</f>
+        <v>1</v>
       </c>
       <c r="E13" s="27" t="n">
-        <f aca="false">COUNTIFS(Blocs!$A$2:$A$179,A13,Blocs!$F$2:$F$179,"&lt;&gt;À tester")</f>
-        <v>0</v>
+        <f aca="false">COUNTIFS(Blocs!$A$2:$A$116,A13,Blocs!$F$2:$F$116,"&lt;&gt;À tester")</f>
+        <v>1</v>
       </c>
       <c r="F13" s="27" t="n">
-        <f aca="false">COUNTIFS(Blocs!$A$2:$A$179,A13,Blocs!$F$2:$F$179,"Oui")</f>
-        <v>0</v>
+        <f aca="false">COUNTIFS(Blocs!$A$2:$A$116,A13,Blocs!$F$2:$F$116,"Oui")</f>
+        <v>1</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="26" t="s">
-        <v>265</v>
+        <v>419</v>
       </c>
       <c r="B14" s="27" t="n">
-        <f aca="false">COUNTIF(Blocs!$A$2:$A$179,A14)</f>
-        <v>8</v>
+        <f aca="false">COUNTIF(Blocs!$A$2:$A$116,A14)</f>
+        <v>2</v>
       </c>
       <c r="C14" s="27" t="n">
-        <f aca="false">COUNTIFS(Blocs!$A$2:$A$179,A14,Blocs!$E$2:$E$179,"&lt;&gt;À tester")</f>
+        <f aca="false">COUNTIFS(Blocs!$A$2:$A$116,A14,Blocs!$E$2:$E$116,"&lt;&gt;À tester")</f>
         <v>0</v>
       </c>
       <c r="D14" s="27" t="n">
-        <f aca="false">COUNTIFS(Blocs!$A$2:$A$179,A14,Blocs!$E$2:$E$179,"Oui")</f>
+        <f aca="false">COUNTIFS(Blocs!$A$2:$A$116,A14,Blocs!$E$2:$E$116,"Oui")</f>
         <v>0</v>
       </c>
       <c r="E14" s="27" t="n">
-        <f aca="false">COUNTIFS(Blocs!$A$2:$A$179,A14,Blocs!$F$2:$F$179,"&lt;&gt;À tester")</f>
+        <f aca="false">COUNTIFS(Blocs!$A$2:$A$116,A14,Blocs!$F$2:$F$116,"&lt;&gt;À tester")</f>
         <v>0</v>
       </c>
       <c r="F14" s="27" t="n">
-        <f aca="false">COUNTIFS(Blocs!$A$2:$A$179,A14,Blocs!$F$2:$F$179,"Oui")</f>
+        <f aca="false">COUNTIFS(Blocs!$A$2:$A$116,A14,Blocs!$F$2:$F$116,"Oui")</f>
         <v>0</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="26" t="s">
-        <v>282</v>
-      </c>
-      <c r="B15" s="27" t="n">
-        <f aca="false">COUNTIF(Blocs!$A$2:$A$179,A15)</f>
-        <v>50</v>
-      </c>
-      <c r="C15" s="27" t="n">
-        <f aca="false">COUNTIFS(Blocs!$A$2:$A$179,A15,Blocs!$E$2:$E$179,"&lt;&gt;À tester")</f>
-        <v>4</v>
-      </c>
-      <c r="D15" s="27" t="n">
-        <f aca="false">COUNTIFS(Blocs!$A$2:$A$179,A15,Blocs!$E$2:$E$179,"Oui")</f>
-        <v>4</v>
-      </c>
-      <c r="E15" s="27" t="n">
-        <f aca="false">COUNTIFS(Blocs!$A$2:$A$179,A15,Blocs!$F$2:$F$179,"&lt;&gt;À tester")</f>
-        <v>4</v>
-      </c>
-      <c r="F15" s="27" t="n">
-        <f aca="false">COUNTIFS(Blocs!$A$2:$A$179,A15,Blocs!$F$2:$F$179,"Oui")</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="26" t="s">
-        <v>401</v>
-      </c>
-      <c r="B16" s="27" t="n">
-        <f aca="false">COUNTIF(Blocs!$A$2:$A$179,A16)</f>
-        <v>2</v>
-      </c>
-      <c r="C16" s="27" t="n">
-        <f aca="false">COUNTIFS(Blocs!$A$2:$A$179,A16,Blocs!$E$2:$E$179,"&lt;&gt;À tester")</f>
-        <v>0</v>
-      </c>
-      <c r="D16" s="27" t="n">
-        <f aca="false">COUNTIFS(Blocs!$A$2:$A$179,A16,Blocs!$E$2:$E$179,"Oui")</f>
-        <v>0</v>
-      </c>
-      <c r="E16" s="27" t="n">
-        <f aca="false">COUNTIFS(Blocs!$A$2:$A$179,A16,Blocs!$F$2:$F$179,"&lt;&gt;À tester")</f>
-        <v>0</v>
-      </c>
-      <c r="F16" s="27" t="n">
-        <f aca="false">COUNTIFS(Blocs!$A$2:$A$179,A16,Blocs!$F$2:$F$179,"Oui")</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="26" t="s">
-        <v>406</v>
-      </c>
-      <c r="B17" s="27" t="n">
-        <f aca="false">COUNTIF(Blocs!$A$2:$A$179,A17)</f>
-        <v>7</v>
-      </c>
-      <c r="C17" s="27" t="n">
-        <f aca="false">COUNTIFS(Blocs!$A$2:$A$179,A17,Blocs!$E$2:$E$179,"&lt;&gt;À tester")</f>
-        <v>1</v>
-      </c>
-      <c r="D17" s="27" t="n">
-        <f aca="false">COUNTIFS(Blocs!$A$2:$A$179,A17,Blocs!$E$2:$E$179,"Oui")</f>
-        <v>1</v>
-      </c>
-      <c r="E17" s="27" t="n">
-        <f aca="false">COUNTIFS(Blocs!$A$2:$A$179,A17,Blocs!$F$2:$F$179,"&lt;&gt;À tester")</f>
-        <v>1</v>
-      </c>
-      <c r="F17" s="27" t="n">
-        <f aca="false">COUNTIFS(Blocs!$A$2:$A$179,A17,Blocs!$F$2:$F$179,"Oui")</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="26" t="s">
-        <v>419</v>
-      </c>
-      <c r="B18" s="27" t="n">
-        <f aca="false">COUNTIF(Blocs!$A$2:$A$179,A18)</f>
-        <v>2</v>
-      </c>
-      <c r="C18" s="27" t="n">
-        <f aca="false">COUNTIFS(Blocs!$A$2:$A$179,A18,Blocs!$E$2:$E$179,"&lt;&gt;À tester")</f>
-        <v>0</v>
-      </c>
-      <c r="D18" s="27" t="n">
-        <f aca="false">COUNTIFS(Blocs!$A$2:$A$179,A18,Blocs!$E$2:$E$179,"Oui")</f>
-        <v>0</v>
-      </c>
-      <c r="E18" s="27" t="n">
-        <f aca="false">COUNTIFS(Blocs!$A$2:$A$179,A18,Blocs!$F$2:$F$179,"&lt;&gt;À tester")</f>
-        <v>0</v>
-      </c>
-      <c r="F18" s="27" t="n">
-        <f aca="false">COUNTIFS(Blocs!$A$2:$A$179,A18,Blocs!$F$2:$F$179,"Oui")</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="28" t="s">
+      <c r="A15" s="28" t="s">
         <v>434</v>
       </c>
-      <c r="B19" s="29" t="n">
-        <f aca="false">SUM(B4:B18)</f>
-        <v>178</v>
-      </c>
-      <c r="C19" s="29" t="n">
-        <f aca="false">SUM(C4:C18)</f>
+      <c r="B15" s="29" t="n">
+        <f aca="false">SUM(B4:B14)</f>
+        <v>115</v>
+      </c>
+      <c r="C15" s="29" t="n">
+        <f aca="false">SUM(C4:C14)</f>
         <v>19</v>
       </c>
-      <c r="D19" s="29" t="n">
-        <f aca="false">SUM(D4:D18)</f>
+      <c r="D15" s="29" t="n">
+        <f aca="false">SUM(D4:D14)</f>
         <v>18</v>
       </c>
-      <c r="E19" s="29" t="n">
-        <f aca="false">SUM(E4:E18)</f>
+      <c r="E15" s="29" t="n">
+        <f aca="false">SUM(E4:E14)</f>
         <v>21</v>
       </c>
-      <c r="F19" s="29" t="n">
-        <f aca="false">SUM(F4:F18)</f>
+      <c r="F15" s="29" t="n">
+        <f aca="false">SUM(F4:F14)</f>
         <v>20</v>
       </c>
     </row>

</xml_diff>